<commit_message>
added definitions to the parameters in all files
</commit_message>
<xml_diff>
--- a/data_in_templates/input_breakthrough_temp.xlsx
+++ b/data_in_templates/input_breakthrough_temp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mohammedfaran/Desktop/python_models/ReactorModels/data_in_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3009DE8-057A-9E4B-8CE0-D3910F97CC76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0D5FF36-B907-964D-80AD-682ACAAA315C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2100" yWindow="2060" windowWidth="26700" windowHeight="15940" activeTab="3" xr2:uid="{BEB422E4-985B-DA42-A0EA-C89047788836}"/>
+    <workbookView xWindow="2100" yWindow="2060" windowWidth="26700" windowHeight="15940" xr2:uid="{BEB422E4-985B-DA42-A0EA-C89047788836}"/>
   </bookViews>
   <sheets>
     <sheet name="breakthrough_parameters" sheetId="5" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
   <si>
     <t xml:space="preserve">time </t>
   </si>
@@ -96,6 +96,107 @@
   </si>
   <si>
     <t>chemical 7</t>
+  </si>
+  <si>
+    <t>definition</t>
+  </si>
+  <si>
+    <t>Volumetric flow rate of water through the packed column. It is the liquid volume passing through the column per unit time.</t>
+  </si>
+  <si>
+    <t>Superficial (empty-bed) velocity of the liquid, calculated as flow rate divided by the column cross-sectional area. It does not correct for the bed porosity.</t>
+  </si>
+  <si>
+    <t>Dimensionless initial mass fraction supplied as a starting condition for the model. Its exact physical interpretation depends on how the selected model uses this field; a value of 0 represents no initial mass of the modeled component when an initially unloaded condition is intended.</t>
+  </si>
+  <si>
+    <t>reference unit</t>
+  </si>
+  <si>
+    <t>required value</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>feed_concentration_sheet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:  Contains the influent/feed concentration of each chemical entering the reactor or treatment column. [M/L^3]</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">effluent_concentration_sheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Contains the measured concentration of each chemical leaving the reactor or treatment column during the experiment.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> [M/L^3]</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>initial_concentration_sheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Contains the concentration of each chemical initially present in the reactor or column before the experiment begins.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> [M/L^3]</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -107,7 +208,7 @@
     <numFmt numFmtId="164" formatCode="0.00000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -155,8 +256,50 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -173,6 +316,11 @@
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -241,7 +389,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -249,9 +397,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -265,6 +410,38 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -600,55 +777,95 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28273D33-CC04-8B4C-B07E-FF186E451A94}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="5" width="130.1640625" customWidth="1"/>
+    <col min="6" max="6" width="14.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="16"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="13"/>
+    </row>
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="20" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+      <c r="E2" s="20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9" t="s">
+      <c r="B3" s="15"/>
+      <c r="C3" s="16" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
+      <c r="D3" s="24"/>
+      <c r="E3" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9" t="s">
+      <c r="B4" s="16"/>
+      <c r="C4" s="16" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="D4" s="24"/>
+      <c r="E4" s="17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="A5" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10" t="s">
+      <c r="B5" s="18"/>
+      <c r="C5" s="18" t="s">
         <v>10</v>
+      </c>
+      <c r="D5" s="24"/>
+      <c r="E5" s="21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E6" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E7" s="25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E8" s="25" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -656,6 +873,7 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -815,422 +1033,422 @@
       <c r="I12" s="4"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="13"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="13"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A23" s="11"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
+      <c r="A23" s="8"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A24" s="11"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
+      <c r="A24" s="8"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="13"/>
+      <c r="A25" s="8"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A26" s="11"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="13"/>
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
+      <c r="A27" s="8"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13"/>
-      <c r="I28" s="13"/>
+      <c r="A28" s="8"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A29" s="11"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="13"/>
+      <c r="A29" s="8"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A30" s="11"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="13"/>
+      <c r="A30" s="8"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A31" s="11"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="13"/>
+      <c r="A31" s="8"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A32" s="11"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A33" s="11"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A34" s="11"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="13"/>
+      <c r="A34" s="8"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A35" s="11"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
+      <c r="A35" s="8"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="13"/>
+      <c r="A36" s="8"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="13"/>
+      <c r="A37" s="8"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="13"/>
+      <c r="A38" s="8"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A39" s="11"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="13"/>
+      <c r="A39" s="8"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A40" s="11"/>
-      <c r="B40" s="11"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
+      <c r="A40" s="8"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A41" s="11"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
-      <c r="H41" s="13"/>
-      <c r="I41" s="13"/>
+      <c r="A41" s="8"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A42" s="11"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
+      <c r="A42" s="8"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="10"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A43" s="11"/>
-      <c r="B43" s="11"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13"/>
-      <c r="H43" s="13"/>
-      <c r="I43" s="13"/>
+      <c r="A43" s="8"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A44" s="11"/>
-      <c r="B44" s="11"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="13"/>
-      <c r="H44" s="13"/>
-      <c r="I44" s="13"/>
+      <c r="A44" s="8"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A45" s="11"/>
-      <c r="B45" s="11"/>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="13"/>
-      <c r="H45" s="13"/>
-      <c r="I45" s="13"/>
+      <c r="A45" s="8"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A46" s="11"/>
-      <c r="B46" s="11"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="13"/>
-      <c r="H46" s="13"/>
-      <c r="I46" s="13"/>
+      <c r="A46" s="8"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+      <c r="I46" s="10"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A47" s="11"/>
-      <c r="B47" s="11"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="13"/>
-      <c r="H47" s="13"/>
-      <c r="I47" s="13"/>
+      <c r="A47" s="8"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+      <c r="I47" s="10"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A48" s="11"/>
-      <c r="B48" s="11"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
+      <c r="A48" s="8"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+      <c r="I48" s="10"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A49" s="11"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="13"/>
-      <c r="F49" s="13"/>
-      <c r="G49" s="13"/>
-      <c r="H49" s="13"/>
-      <c r="I49" s="13"/>
+      <c r="A49" s="8"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="10"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" s="11"/>
-      <c r="B50" s="11"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="13"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="13"/>
-      <c r="G50" s="13"/>
-      <c r="H50" s="13"/>
-      <c r="I50" s="13"/>
+      <c r="A50" s="8"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+      <c r="I50" s="10"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
@@ -1405,422 +1623,422 @@
       <c r="I12" s="4"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="13"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="13"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A23" s="11"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
+      <c r="A23" s="8"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A24" s="11"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
+      <c r="A24" s="8"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="13"/>
+      <c r="A25" s="8"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A26" s="11"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="13"/>
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A27" s="11"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
+      <c r="A27" s="8"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13"/>
-      <c r="I28" s="13"/>
+      <c r="A28" s="8"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A29" s="11"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="13"/>
+      <c r="A29" s="8"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A30" s="11"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="13"/>
+      <c r="A30" s="8"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A31" s="11"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="13"/>
+      <c r="A31" s="8"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A32" s="11"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A33" s="11"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A34" s="11"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="13"/>
+      <c r="A34" s="8"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A35" s="11"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
+      <c r="A35" s="8"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="13"/>
+      <c r="A36" s="8"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A37" s="11"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="13"/>
+      <c r="A37" s="8"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="13"/>
+      <c r="A38" s="8"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A39" s="11"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="13"/>
+      <c r="A39" s="8"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A40" s="11"/>
-      <c r="B40" s="11"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
+      <c r="A40" s="8"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A41" s="11"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
-      <c r="H41" s="13"/>
-      <c r="I41" s="13"/>
+      <c r="A41" s="8"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A42" s="11"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
+      <c r="A42" s="8"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="10"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A43" s="11"/>
-      <c r="B43" s="11"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13"/>
-      <c r="H43" s="13"/>
-      <c r="I43" s="13"/>
+      <c r="A43" s="8"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A44" s="11"/>
-      <c r="B44" s="11"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="13"/>
-      <c r="H44" s="13"/>
-      <c r="I44" s="13"/>
+      <c r="A44" s="8"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A45" s="11"/>
-      <c r="B45" s="11"/>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="13"/>
-      <c r="H45" s="13"/>
-      <c r="I45" s="13"/>
+      <c r="A45" s="8"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A46" s="11"/>
-      <c r="B46" s="11"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="13"/>
-      <c r="H46" s="13"/>
-      <c r="I46" s="13"/>
+      <c r="A46" s="8"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+      <c r="I46" s="10"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A47" s="11"/>
-      <c r="B47" s="11"/>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="13"/>
-      <c r="H47" s="13"/>
-      <c r="I47" s="13"/>
+      <c r="A47" s="8"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+      <c r="I47" s="10"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A48" s="11"/>
-      <c r="B48" s="11"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
+      <c r="A48" s="8"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+      <c r="I48" s="10"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A49" s="11"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="13"/>
-      <c r="F49" s="13"/>
-      <c r="G49" s="13"/>
-      <c r="H49" s="13"/>
-      <c r="I49" s="13"/>
+      <c r="A49" s="8"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="10"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" s="11"/>
-      <c r="B50" s="11"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="13"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="13"/>
-      <c r="G50" s="13"/>
-      <c r="H50" s="13"/>
-      <c r="I50" s="13"/>
+      <c r="A50" s="8"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+      <c r="I50" s="10"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
@@ -1848,7 +2066,7 @@
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -1875,13 +2093,13 @@
       <c r="J1" s="5"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>

</xml_diff>